<commit_message>
Remove answer-control terminology from workbook
</commit_message>
<xml_diff>
--- a/artifacts/关键标准答案.xlsx
+++ b/artifacts/关键标准答案.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="交付物答案清单" sheetId="1" r:id="Rdeef1454af1449a5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="固定字段答案" sheetId="2" r:id="R457e9bc3358a4006"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="固定集合答案" sheetId="3" r:id="Rf8d42486f2264841"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="固定数值答案" sheetId="4" r:id="R631866e18ba94167"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="允许变体答案" sheetId="5" r:id="R0b3e7625243d43d3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="交付物答案清单" sheetId="1" r:id="R818318615f544803"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="固定字段答案" sheetId="2" r:id="R8a5602e8844346a6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="固定集合答案" sheetId="3" r:id="Re701d88103784041"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="固定数值答案" sheetId="4" r:id="R2951f0f56ab048ec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="允许变体答案" sheetId="5" r:id="R4daa8ede61d94ac8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -634,7 +634,7 @@
     </x:row>
     <x:row r="6" ht="92" customHeight="1">
       <x:c r="A6" s="9" t="str">
-        <x:v>reference_members</x:v>
+        <x:v>browser_delivery_paths</x:v>
       </x:c>
       <x:c r="B6" s="9" t="str">
         <x:v>output/playwright.config.ts、output/tests/subscription_settings.spec.ts、output/reports/settings_state_report.csv、output/reports/save_rollback_report.csv、output/reports/keyboard_focus_report.csv</x:v>
@@ -643,7 +643,7 @@
         <x:v>相对路径逐字匹配</x:v>
       </x:c>
       <x:c r="D6" s="9" t="str">
-        <x:v>reference.zip成员</x:v>
+        <x:v>任务Prompt声明的浏览器交付路径</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>